<commit_message>
Corregir bug de tendencia para sucursales sin datos en el trimestre reciente
Las sucursales que dejaron de reportar (o son nuevas) se etiquetaban
por error como "Estable" al comparar trimestres, porque la diferencia
daba NaN y el chequeo de umbral la dejaba caer en el caso por defecto.
Ahora se distinguen explicitamente como "Sin datos recientes" o
"Sucursal nueva", evitando subestimar el numero real de sucursales
con problemas de seguimiento. Se actualizan dashboard, reporte
ejecutivo y Excel para reflejar las nuevas categorias de tendencia.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/Analisis_Metas_Calzapato.xlsx
+++ b/reports/Analisis_Metas_Calzapato.xlsx
@@ -573,7 +573,7 @@
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
@@ -906,7 +906,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1624,7 +1624,7 @@
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>➡️ Estable</t>
+          <t>⚠️ Sin datos recientes</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">

</xml_diff>